<commit_message>
Setup Database môi trường Dev
</commit_message>
<xml_diff>
--- a/DS CHỨC NĂNG.xlsx
+++ b/DS CHỨC NĂNG.xlsx
@@ -8,29 +8,6 @@
   <definedNames/>
   <calcPr/>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
-  <authors>
-    <author>tc={afb1c72b-452b-46de-b39d-c594d88527a2}</author>
-  </authors>
-  <commentList>
-    <comment authorId="0" xr:uid="{afb1c72b-452b-46de-b39d-c594d88527a2}" ref="D8">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	cái này đang thấy nó là tài khoản tiết kiệm thôi
-Reply:
-	tao đang muốn nó là tài khoản liên kết với số dư update của từng tháng khi mình nhận thu nhập và chi tiêu
-1 total reaction
-Liên Hoàng Ngọc reacted with 🥰 at 08/27/2026, 4:06 AM UTC
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -284,18 +261,12 @@
 </styleSheet>
 </file>
 
-<file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
-<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Diệu Linh Vũ Thị" id="{cf1e58c3-bab9-452f-a73a-2984fddfc343}" providerId="google-sheets"/>
-</x18tc:personList>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -492,19 +463,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="D8" dT="2026-08-21T07:52:00.00" personId="{cf1e58c3-bab9-452f-a73a-2984fddfc343}" id="{afb1c72b-452b-46de-b39d-c594d88527a2}" done="0">
-    <x18tc:text xml:space="preserve">cái này đang thấy nó là tài khoản tiết kiệm thôi</x18tc:text>
-  </x18tc:threadedComment>
-  <x18tc:threadedComment ref="D8" dT="2026-08-21T07:52:58.00" personId="{cf1e58c3-bab9-452f-a73a-2984fddfc343}" id="{dc1ea4fd-0ef2-4101-aecb-b08b5bdf09cd}" parentId="{afb1c72b-452b-46de-b39d-c594d88527a2}">
-    <x18tc:text xml:space="preserve">tao đang muốn nó là tài khoản liên kết với số dư update của từng tháng khi mình nhận thu nhập và chi tiêu
-1 total reaction
-Liên Hoàng Ngọc reacted with 🥰 at 08/27/2026, 4:06 AM UTC</x18tc:text>
-  </x18tc:threadedComment>
-</x18tc:ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
@@ -1479,7 +1437,6 @@
       <formula1>"Cao,Trung bình"</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId4"/>
-  <legacyDrawing r:id="rId5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>